<commit_message>
Update Case 1 and 2 with cosmetic edit
</commit_message>
<xml_diff>
--- a/Compare-R1-SW1-4-Cases.xlsx
+++ b/Compare-R1-SW1-4-Cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cf954df90cd41547/Documents/Cisco-CCNA-200-301/HY-Portfolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="138" documentId="13_ncr:1_{E28D1B89-7AC4-42B0-884C-B2A303006F34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FEA2667-7712-4951-8E0C-7510778292D4}"/>
+  <xr:revisionPtr revIDLastSave="214" documentId="13_ncr:1_{E28D1B89-7AC4-42B0-884C-B2A303006F34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D65DB32-D203-4810-AEC3-4A8931A4339D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="R1" sheetId="1" r:id="rId1"/>
@@ -61,19 +61,7 @@
     <t>ipv6 unicast-routing</t>
   </si>
   <si>
-    <t>ip route 192.168.0.0 255.255.0.0 10.0.0.2</t>
-  </si>
-  <si>
     <t>ipv6 route 2001:db8:0::/48 2001:db8:0:0::2</t>
-  </si>
-  <si>
-    <t>! R1 -- SW1
-! gig0/0/1 is built-in L3 port 
-interface gigabitethernet0/0/1
- description R1 -- SW1 
- ip   address 10.0.0.1 255.255.255.252
- ipv6 address 2001:db8:0:0::1/64
- ipv6 address fe80::1         link-local</t>
   </si>
   <si>
     <t>! R1 -- ISP
@@ -92,23 +80,6 @@
  ipv6 address fe80::1         link-local</t>
   </si>
   <si>
-    <t>interface gigabitethernet0/0/1
- description R1 -- SW1 
- no ip   address 
- no ipv6 address</t>
-  </si>
-  <si>
-    <t>! R1 -- SW1
-! gig0/0/1 is L3 ports
-! SW1 is L2 2960-24TT switch
-interface gigabitethernet0/0/1.10
- description R1 -- SW1 (VLAN 10: Eng)
- encapsulation dot1q 10
- ip   address 192.168.10.1 255.255.255.0
- ipv6 address 2001:db8:0:10::1/64
- ipv6 address fe80::1         link-local</t>
-  </si>
-  <si>
     <t>interface gigabitethernet0/0/1.20
  description R1 -- SW1 (VLAN 20: Sales) 
  encapsulation dot1q 20
@@ -125,15 +96,6 @@
  ipv6 address fe80::1         link-local</t>
   </si>
   <si>
-    <t>! VLAN 99 Management default gateway 192.168.99.1
-interface gigabitethernet0/0/1.99
- description R1 -- SW1 (VLAN 99: Management)
- encapsulation dot1q 99
- ip   address 192.168.99.1 255.255.255.0
- ipv6 address 2001:db8:0:99::1/64
- ipv6 address fe80::1         link-local</t>
-  </si>
-  <si>
     <t>! 2. Fix the Native VLAN Mismatch on the Trunk
 interface gigabitethernet0/0/1.199
  description R1 -- SW1 (VLAN 199: Native)
@@ -167,12 +129,6 @@
 vlan 30 name Admin
 vlan 99 name Management
 vlan 199 name Native</t>
-  </si>
-  <si>
-    <t>interface vlan 99
- ip address 192.168.99.101 255.255.255.0
- ipv6 address 2001:db8:0:99::101/64
- ipv6 address fe80::1            link-local</t>
   </si>
   <si>
     <t>interface vlan 30
@@ -205,10 +161,6 @@
   <si>
     <t>vlan database
 vlan 999 name Transit_To_SW1</t>
-  </si>
-  <si>
-    <t>! 4. Static Routes pointing to SW1
-ip route 192.168.0.0 255.255.0.0 10.0.0.2</t>
   </si>
   <si>
     <t>! 2. Create the SVI to hold the IP address
@@ -271,23 +223,6 @@
  ipv6 address fe80::21         link-local</t>
   </si>
   <si>
-    <t>! Static route pointing to R1 for internet traffic
-ip route 0.0.0.0 0.0.0.0 10.0.0.1
-ipv6 route ::/0 2001:db8:0:0::1</t>
-  </si>
-  <si>
-    <t>! SW1 -- R1
-! gig1/0/1 is L3 ports
-! The link to R1 becomes a true Layer 3 port
-interface gigabitethernet1/0/1
- description SW1 -- R1 
- no switchport
- no cdp enable
- ip   address 10.0.0.2 255.255.255.252
- ipv6 address 2001:db8:0:0::2/64
- ipv6 address fe80::21        link-local</t>
-  </si>
-  <si>
     <t>! SW1 -- SW2
 ! gig1/0/2 to SW2 L2 Switch 2960-24TT
 interface gigabitethernet1/0/2
@@ -335,10 +270,6 @@
 name Native</t>
   </si>
   <si>
-    <t>! Point SW1 to R1
-ip default-gateway 192.168.99.101</t>
-  </si>
-  <si>
     <t>! SW1 -- R1
 ! gig0/1 is L2 ports
 interface gigabitethernet0/1
@@ -395,20 +326,6 @@
 Why loopback OK? </t>
   </si>
   <si>
-    <t>ip route 0.0.0.0 0.0.0.0 10.0.0.1
-ipv6 route ::/0 2001:db8:0:0::1</t>
-  </si>
-  <si>
-    <t>! SW1 -- R1
-! gig1/0/1 is L3 ports
-interface gigabitethernet1/0/1
- description SW1 -- R1 
- no switchport
- ip   address 10.0.0.2 255.255.255.252
- ipv6 address 2001:db8:0:0::2/64
- ipv6 address fe80::21        link-local</t>
-  </si>
-  <si>
     <t>! SW1 -- SW3
 ! gig1/0/3 to SW3 L2 Switch 2960-24TT
 interface gigabitethernet1/0/3
@@ -421,18 +338,6 @@
   <si>
     <t>This is L3 Switch 3650-24PS
 Loopback As Expected</t>
-  </si>
-  <si>
-    <t>! 2. Configure Default Gateway (points to R1's subinterface IP)
-ip default-gateway 192.168.99.1</t>
-  </si>
-  <si>
-    <t>! 1. Create SVI for SW1 Management IP
-interface vlan 99
- description SW1 Management SVI
- ip address 192.168.99.11 255.255.255.0
- ipv6 address 2001:db8:0:99::11/64
- ipv6 address fe80::21 link-local</t>
   </si>
   <si>
     <t>! SW1 -- R1
@@ -809,12 +714,332 @@
  switchport trunk native vlan 199
  switchport trunk allowed vlan 10,20,30,99</t>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">! SW1 -- R1
+! gig1/0/1 is L3 ports
+interface gigabitethernet1/0/1
+ description SW1 -- R1 
+ no switchport
+ ip   address </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>10.0.0.2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 255.255.255.252
+ ipv6 address 2001:db8:0:0::2/64
+ ipv6 address fe80::21        link-local</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">! R1 -- SW1
+! gig0/0/1 is built-in L3 port 
+interface gigabitethernet0/0/1
+ description R1 -- SW1 
+ ip   address </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>10.0.0.1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 255.255.255.252
+ ipv6 address 2001:db8:0:0::1/64
+ ipv6 address fe80::1         link-local</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">! Static route pointing to R1 for internet traffic
+ip route 0.0.0.0 0.0.0.0 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>10.0.0.1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ipv6 route ::/0 2001:db8:0:0::1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">! SW1 -- R1
+! gig1/0/1 is L3 ports
+! The link to R1 becomes a true Layer 3 port
+interface gigabitethernet1/0/1
+ description SW1 -- R1 
+ no switchport
+ no cdp enable
+ ip   address </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>10.0.0.2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 255.255.255.252
+ ipv6 address 2001:db8:0:0::2/64
+ ipv6 address fe80::21        link-local</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ip route 192.168.0.0 255.255.0.0 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>10.0.0.2</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ip route 0.0.0.0 0.0.0.0 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>10.0.0.1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ipv6 route ::/0 2001:db8:0:0::1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">! 4. Static Routes pointing to SW1
+ip route 192.168.0.0 255.255.0.0 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>10.0.0.2</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">! VLAN 99 Management default gateway 192.168.99.1
+interface gigabitethernet0/0/1.99
+ description R1 -- SW1 (VLAN 99: Management)
+ encapsulation dot1q 99
+ ip   address </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>192.168.99.1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 255.255.255.0
+ ipv6 address 2001:db8:0:99::1/64
+ ipv6 address fe80::1         link-local</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">interface vlan 99
+ ip address </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>192.168.99.101</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 255.255.255.0
+ ipv6 address 2001:db8:0:99::101/64
+ ipv6 address fe80::1            link-local</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">! 2. Configure Default Gateway (points to R1's subinterface IP)
+ip default-gateway </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>192.168.99.1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">! Point SW1 to R1
+ip default-gateway </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>192.168.99.101</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">! 1. Create SVI for SW1 Management IP
+interface vlan 99
+ description SW1 Management SVI
+ ip address </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>192.168.99.11</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 255.255.255.0
+ ipv6 address 2001:db8:0:99::11/64
+ ipv6 address fe80::21 link-local</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">
+interface gigabitethernet0/0/1.10
+ description R1 -- SW1 (VLAN 10: Eng)
+ encapsulation dot1q 10
+ ip   address 192.168.10.1 255.255.255.0
+ ipv6 address 2001:db8:0:10::1/64
+ ipv6 address fe80::1         link-local</t>
+  </si>
+  <si>
+    <t>! R1 -- SW1
+! R1 gig0/0/1 is built-in L3 ports
+! SW1 is L2 2960-24TT switch
+interface gigabitethernet0/0/1
+ description R1 -- SW1 
+ no ip   address 
+ no ipv6 address</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -822,13 +1047,39 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -843,9 +1094,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1128,7 +1386,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="41.21875" customWidth="1"/>
@@ -1213,25 +1471,25 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>9</v>
+      <c r="A7" s="3" t="s">
+        <v>102</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>31</v>
+        <v>89</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -1239,115 +1497,114 @@
     </row>
     <row r="10" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="129.6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
-      <c r="B12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>28</v>
-      </c>
+      <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
+    <row r="13" spans="1:5" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>99</v>
+      </c>
       <c r="B13" s="1" t="s">
-        <v>16</v>
+        <v>111</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-    </row>
-    <row r="14" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="1" t="s">
-        <v>17</v>
+        <v>110</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="1"/>
+        <v>13</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>20</v>
+      </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1" t="s">
+      <c r="B17" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C17" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18" spans="1:5" ht="92.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
+      <c r="B18" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
+      <c r="D19" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
@@ -1356,68 +1613,82 @@
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="B23" s="1" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D23" s="1"/>
-    </row>
-    <row r="24" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B24" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D24" s="1"/>
-    </row>
-    <row r="25" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
       <c r="B25" s="1" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D25" s="1"/>
     </row>
     <row r="26" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B26" s="1" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="D26" s="1"/>
     </row>
-    <row r="28" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B27" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" s="1"/>
+    </row>
+    <row r="28" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B28" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="C28" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D28" s="1"/>
+    </row>
+    <row r="30" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="C30" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1429,7 +1700,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F93DA400-1F27-4D46-ABD8-A59639C7CD46}">
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="47.5546875" customWidth="1"/>
@@ -1473,7 +1744,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1490,262 +1761,290 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>8</v>
+    <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" ht="153.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B8" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>47</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
       <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
-    </row>
-    <row r="10" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B13" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="144" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="E10" s="1" t="s">
+      <c r="D30" s="1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="144" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C20" s="1" t="s">
+      <c r="E30" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E22" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
+      <c r="D31" s="1"/>
+      <c r="E31" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A50" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1763,7 +2062,7 @@
     <col min="1" max="1" width="38.44140625" customWidth="1"/>
     <col min="2" max="2" width="41.21875" customWidth="1"/>
     <col min="3" max="3" width="38.44140625" customWidth="1"/>
-    <col min="4" max="4" width="34.5546875" customWidth="1"/>
+    <col min="4" max="4" width="43.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -1824,16 +2123,16 @@
     </row>
     <row r="7" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1846,10 +2145,10 @@
   <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="32.5546875" customWidth="1"/>
-    <col min="3" max="3" width="32.77734375" customWidth="1"/>
-    <col min="4" max="4" width="31.33203125" customWidth="1"/>
+    <col min="1" max="1" width="35.44140625" customWidth="1"/>
+    <col min="2" max="2" width="42" customWidth="1"/>
+    <col min="3" max="3" width="40.21875" customWidth="1"/>
+    <col min="4" max="4" width="38" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -1896,86 +2195,86 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="D5" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>81</v>
-      </c>
       <c r="C13" s="1" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="144" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>78</v>
-      </c>
       <c r="D17" s="1" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -2038,83 +2337,83 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="D5" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>85</v>
-      </c>
       <c r="D13" s="1" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2177,86 +2476,86 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="D5" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>